<commit_message>
Week 2: Active Members, Offboarded, Projects, Training Tabs Work.
</commit_message>
<xml_diff>
--- a/Data/HRData.xlsx
+++ b/Data/HRData.xlsx
@@ -1,23 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\HROnboardingApp\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B234EFB-5125-4529-AFC1-EAAB3B866739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2583236-67EB-4315-9355-923B324B130D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{30C4A489-88FD-4F42-90A7-1AA7E270F543}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{30C4A489-88FD-4F42-90A7-1AA7E270F543}"/>
   </bookViews>
   <sheets>
-    <sheet name="Candidates" sheetId="2" r:id="rId1"/>
-    <sheet name="Users" sheetId="3" r:id="rId2"/>
-    <sheet name="Training" sheetId="4" r:id="rId3"/>
-    <sheet name="OnboardingSteps" sheetId="5" r:id="rId4"/>
-    <sheet name="OnboardingProcess" sheetId="6" r:id="rId5"/>
+    <sheet name="Users" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,150 +39,51 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>ROVO(Y/N)</t>
-  </si>
-  <si>
-    <t>CandidateID</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>Role</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>JoinDate</t>
-  </si>
-  <si>
-    <t>Team</t>
-  </si>
-  <si>
     <t>UserID</t>
   </si>
   <si>
     <t>PasswordHash</t>
   </si>
   <si>
-    <t>TrainingID</t>
-  </si>
-  <si>
-    <t>CandidateId</t>
-  </si>
-  <si>
-    <t>DueDate</t>
-  </si>
-  <si>
-    <t>CompletionDate</t>
-  </si>
-  <si>
-    <t>StepID</t>
-  </si>
-  <si>
-    <t>TeamName</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>StepName</t>
-  </si>
-  <si>
-    <t>StepOrder</t>
-  </si>
-  <si>
-    <t>ProcessID</t>
-  </si>
-  <si>
-    <t>CompletedDate</t>
-  </si>
-  <si>
-    <t>Rohan K</t>
-  </si>
-  <si>
-    <t>rohan@test.com</t>
-  </si>
-  <si>
-    <t>.Net Dev</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>FW</t>
-  </si>
-  <si>
-    <t>Kanika R</t>
-  </si>
-  <si>
-    <t>Raskan@test.com</t>
-  </si>
-  <si>
-    <t>Cloud Admin</t>
-  </si>
-  <si>
-    <t>InActive</t>
-  </si>
-  <si>
-    <t>Datadog(Y/N)</t>
-  </si>
-  <si>
-    <t>AKS Trained(Y/N)</t>
-  </si>
-  <si>
-    <t>AI Fluency(Y/N)</t>
-  </si>
-  <si>
-    <t>Claude 101(Y/N)</t>
-  </si>
-  <si>
-    <t>AZ900(Y/N)</t>
-  </si>
-  <si>
-    <t>Other Certifications(Y/N)</t>
-  </si>
-  <si>
-    <t>CoPilot Training(Y/N)</t>
-  </si>
-  <si>
-    <t>FW 2.0</t>
-  </si>
-  <si>
-    <t>admin</t>
-  </si>
-  <si>
-    <t>admin123</t>
-  </si>
-  <si>
     <t>Admin</t>
   </si>
   <si>
-    <t>user1</t>
-  </si>
-  <si>
-    <t>user123</t>
-  </si>
-  <si>
     <t>User</t>
   </si>
   <si>
-    <t>user2</t>
-  </si>
-  <si>
-    <t>user456</t>
-  </si>
-  <si>
     <t>Isactive</t>
   </si>
   <si>
     <t>UserName</t>
+  </si>
+  <si>
+    <t>tmadiya@deloitte.com</t>
+  </si>
+  <si>
+    <t>karastogi@deloitte.com</t>
+  </si>
+  <si>
+    <t>kmullangi@deloitte.com</t>
+  </si>
+  <si>
+    <t>rohankulkarni@deloitte.com</t>
+  </si>
+  <si>
+    <t>rohan@2005</t>
+  </si>
+  <si>
+    <t>Admin@123</t>
+  </si>
+  <si>
+    <t>User@123</t>
+  </si>
+  <si>
+    <t>Admin2@123</t>
   </si>
 </sst>
 </file>
@@ -237,11 +134,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -576,133 +472,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{358897FF-3897-4B6D-8A0F-DEA84C78DC28}">
-  <dimension ref="A1:G3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11FB81B8-A234-4EA6-8FB5-B1AA8CB50C92}">
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.7265625" customWidth="1"/>
-    <col min="3" max="3" width="16.26953125" customWidth="1"/>
-    <col min="4" max="4" width="14.26953125" customWidth="1"/>
-    <col min="6" max="6" width="10.08984375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>211</v>
-      </c>
-      <c r="B2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="3">
-        <v>46054</v>
-      </c>
-      <c r="G2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>212</v>
-      </c>
-      <c r="B3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" s="3">
-        <v>46053</v>
-      </c>
-      <c r="G3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{B8141A83-D91E-4C9B-9873-9A8255DDE57D}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{FFEC6C19-BD4A-47DA-ACD1-C81D533079EC}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11FB81B8-A234-4EA6-8FB5-B1AA8CB50C92}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="9.81640625" customWidth="1"/>
+    <col min="2" max="2" width="25.1796875" customWidth="1"/>
     <col min="3" max="3" width="13.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>46</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" t="s">
-        <v>39</v>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -712,165 +518,64 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" t="s">
-        <v>42</v>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="E3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" t="s">
-        <v>45</v>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22F4D1E4-8CDD-4268-BC2F-E6F9377D4BA2}">
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="9.90625" customWidth="1"/>
-    <col min="2" max="3" width="11.36328125" customWidth="1"/>
-    <col min="4" max="4" width="15.08984375" customWidth="1"/>
-    <col min="5" max="5" width="11.36328125" customWidth="1"/>
-    <col min="6" max="6" width="15.26953125" customWidth="1"/>
-    <col min="7" max="7" width="15.81640625" customWidth="1"/>
-    <col min="8" max="8" width="13.54296875" customWidth="1"/>
-    <col min="9" max="9" width="23.36328125" customWidth="1"/>
-    <col min="10" max="10" width="17.7265625" customWidth="1"/>
-    <col min="12" max="12" width="14.26953125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>5</v>
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A39430F7-7ECF-4A8C-8A31-042445403756}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="10.453125" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="11.81640625" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89F9B618-8BC8-49DD-B7A7-74400FF462D0}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="10.90625" customWidth="1"/>
-    <col min="2" max="2" width="11.36328125" customWidth="1"/>
-    <col min="4" max="4" width="14.26953125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{CB67DBA6-7790-4EB6-A889-D8199AF24807}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{C932378A-B275-4CEC-A00E-99313C6EB076}"/>
+    <hyperlink ref="B3" r:id="rId3" xr:uid="{A262B80F-57BE-4C5A-A429-CBBED04D16D2}"/>
+    <hyperlink ref="C3" r:id="rId4" xr:uid="{2EFD2651-4C7A-4AE5-82B2-E03C59259980}"/>
+    <hyperlink ref="B4" r:id="rId5" xr:uid="{12C7EBED-978A-4619-A702-E06BC6A519E3}"/>
+    <hyperlink ref="C4" r:id="rId6" xr:uid="{21F07870-B7E9-4702-AD37-88EB63A04394}"/>
+    <hyperlink ref="B5" r:id="rId7" xr:uid="{2BEB238D-E44F-4C62-9381-656F01486485}"/>
+    <hyperlink ref="C5" r:id="rId8" xr:uid="{AD0B8348-BA58-4245-9CF6-4415EA391380}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Week 3 frontend in progress - backend complete, fixing UI issues.
</commit_message>
<xml_diff>
--- a/Data/HRData.xlsx
+++ b/Data/HRData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\HROnboardingApp\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2583236-67EB-4315-9355-923B324B130D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43273B40-DBFA-4F63-BCC0-5A698D4753D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{30C4A489-88FD-4F42-90A7-1AA7E270F543}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{30C4A489-88FD-4F42-90A7-1AA7E270F543}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>Role</t>
   </si>
@@ -62,9 +62,6 @@
     <t>UserName</t>
   </si>
   <si>
-    <t>tmadiya@deloitte.com</t>
-  </si>
-  <si>
     <t>karastogi@deloitte.com</t>
   </si>
   <si>
@@ -84,6 +81,12 @@
   </si>
   <si>
     <t>Admin2@123</t>
+  </si>
+  <si>
+    <t>tmadiya1@deloitte.com</t>
+  </si>
+  <si>
+    <t>rahullot@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -473,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11FB81B8-A234-4EA6-8FB5-B1AA8CB50C92}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="25.1796875" customWidth="1"/>
@@ -502,10 +505,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
         <v>3</v>
@@ -519,10 +522,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
         <v>4</v>
@@ -536,10 +539,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
         <v>3</v>
@@ -553,16 +556,33 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>12345</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -575,6 +595,7 @@
     <hyperlink ref="C4" r:id="rId6" xr:uid="{21F07870-B7E9-4702-AD37-88EB63A04394}"/>
     <hyperlink ref="B5" r:id="rId7" xr:uid="{2BEB238D-E44F-4C62-9381-656F01486485}"/>
     <hyperlink ref="C5" r:id="rId8" xr:uid="{AD0B8348-BA58-4245-9CF6-4415EA391380}"/>
+    <hyperlink ref="B6" r:id="rId9" xr:uid="{E45C4BC7-5A91-42B8-AACE-05029C11CC76}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Week 3 major progress
</commit_message>
<xml_diff>
--- a/Data/HRData.xlsx
+++ b/Data/HRData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\HROnboardingApp\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43273B40-DBFA-4F63-BCC0-5A698D4753D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B48A3F-1981-4757-B25A-4320B9841C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{30C4A489-88FD-4F42-90A7-1AA7E270F543}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{30C4A489-88FD-4F42-90A7-1AA7E270F543}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>Role</t>
   </si>
@@ -83,10 +83,7 @@
     <t>Admin2@123</t>
   </si>
   <si>
-    <t>tmadiya1@deloitte.com</t>
-  </si>
-  <si>
-    <t>rahullot@gmail.com</t>
+    <t>tmadiya@deloitte.com</t>
   </si>
 </sst>
 </file>
@@ -569,21 +566,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6">
-        <v>12345</v>
-      </c>
-      <c r="D6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" t="b">
-        <v>1</v>
-      </c>
+      <c r="B6" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -595,7 +578,6 @@
     <hyperlink ref="C4" r:id="rId6" xr:uid="{21F07870-B7E9-4702-AD37-88EB63A04394}"/>
     <hyperlink ref="B5" r:id="rId7" xr:uid="{2BEB238D-E44F-4C62-9381-656F01486485}"/>
     <hyperlink ref="C5" r:id="rId8" xr:uid="{AD0B8348-BA58-4245-9CF6-4415EA391380}"/>
-    <hyperlink ref="B6" r:id="rId9" xr:uid="{E45C4BC7-5A91-42B8-AACE-05029C11CC76}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>